<commit_message>
Khanhnq: new feature daily schdule
</commit_message>
<xml_diff>
--- a/files/Daily plan.xlsx
+++ b/files/Daily plan.xlsx
@@ -121,16 +121,16 @@
     <t>Take shower</t>
   </si>
   <si>
-    <t>20:30-22:00</t>
+    <t>20:30-21:30</t>
   </si>
   <si>
     <t>Read book</t>
   </si>
   <si>
-    <t>22:00-22:30</t>
-  </si>
-  <si>
-    <t>23:26-00:00</t>
+    <t>21:30-22:00</t>
+  </si>
+  <si>
+    <t>22:00-00:00</t>
   </si>
   <si>
     <t>Free time</t>
@@ -1161,20 +1161,20 @@
       <c r="B15" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="9" t="s">
-        <v>36</v>
+      <c r="C15" s="11" t="s">
+        <v>18</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="E15" s="9" t="s">
-        <v>36</v>
+      <c r="E15" s="11" t="s">
+        <v>18</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="G15" s="9" t="s">
-        <v>36</v>
+      <c r="G15" s="11" t="s">
+        <v>18</v>
       </c>
       <c r="H15" s="9" t="s">
         <v>36</v>

</xml_diff>